<commit_message>
fix: close N writeback parity gaps
</commit_message>
<xml_diff>
--- a/backend/wp_templates/N/N5 所得税费用.xlsx
+++ b/backend/wp_templates/N/N5 所得税费用.xlsx
@@ -8190,7 +8190,7 @@
         <v/>
       </c>
       <c r="D11" s="514">
-        <f>SUM(D5:N16)</f>
+        <f>SUM(D12:D16)</f>
         <v/>
       </c>
       <c r="E11" s="514">
@@ -8211,7 +8211,7 @@
       <c r="C12" s="516" t="n"/>
       <c r="D12" s="517" t="n"/>
       <c r="E12" s="518">
-        <f>C12+N5</f>
+        <f>C12+D12</f>
         <v/>
       </c>
       <c r="F12" s="289" t="n"/>
@@ -10511,7 +10511,7 @@
       <c r="F12" s="539" t="n"/>
       <c r="G12" s="539" t="n"/>
       <c r="H12" s="540">
-        <f>C12-B12+N5-E12-F12+G12</f>
+        <f>C12-B12+D12-E12-F12+G12</f>
         <v/>
       </c>
       <c r="I12" s="539" t="n"/>

</xml_diff>